<commit_message>
Access guide: one-click "Open" jumps to the view with LOB pre-selected
Each guide row gets an Open button that switches the Data Explorer to that
report view and pre-selects the table's line of business / statement, then opens
the filter modal so the user only picks the entity (+ metric/year). Guide xlsx
gains hidden Dimension/Pick columns to drive this; the visible download stays
the clean 5-column sheet.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge_base/IRIS_Handbook_Access_Guide.xlsx
+++ b/knowledge_base/IRIS_Handbook_Access_Guide.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -434,6 +434,8 @@
     <col width="64" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="90" customWidth="1" min="5" max="5"/>
+    <col hidden="1" width="13" customWidth="1" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,6 +464,16 @@
           <t>How to Access (filter path)</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Dimension</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pick</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -489,6 +501,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -516,6 +538,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -543,6 +575,12 @@
           <t>Industry-wise View → pick Sector → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -570,6 +608,16 @@
           <t>State-wise View → pick State → Line of Business = «Life» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -597,6 +645,16 @@
           <t>State-wise View → pick State → Line of Business = «Individual New Business (Life)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Individual New Business (Life)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -624,6 +682,16 @@
           <t>State-wise View → pick State → Line of Business = «Life» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -651,6 +719,16 @@
           <t>State-wise View → pick State → Line of Business = «Group New Business (Life)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Group New Business (Life)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -678,6 +756,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -705,6 +793,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «In-Force Policies» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>In-Force Policies</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -732,6 +830,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «In-Force Sum Assured» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>In-Force Sum Assured</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -759,6 +867,12 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «the plan / category (Linked, Non-Linked, ULIP, Traditional, Individual/Group)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -786,6 +900,12 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «the plan / category (Linked, Non-Linked, ULIP, Traditional, Individual/Group)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -813,6 +933,16 @@
           <t>Industry-wise View → pick Sector → Line of Business = «Individual Death Claims» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Individual Death Claims</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -840,6 +970,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Individual Death Claims» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Individual Death Claims</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -867,6 +1007,16 @@
           <t>Industry-wise View → pick Sector → Line of Business = «Group Death Claims» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Group Death Claims</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -894,6 +1044,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Group Death Claims» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Group Death Claims</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -921,6 +1081,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Death Claim Settlement Duration - Individual» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Death Claim Settlement Duration - Individual</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -948,6 +1118,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Death Claim Settlement Duration - Group» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Death Claim Settlement Duration - Group</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -975,6 +1155,16 @@
           <t>Industry-wise View → pick Sector → Line of Business = «Investments (AUM)» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Investments (AUM)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1002,6 +1192,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1029,6 +1229,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1056,6 +1266,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Policyholders Account</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1083,6 +1303,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Shareholders Account</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1110,6 +1340,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1137,6 +1377,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Lapsed / Forfeited Policies (Non-Linked)» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Lapsed / Forfeited Policies (Non-Linked)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1164,6 +1414,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Persistency» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Persistency</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1191,6 +1451,16 @@
           <t>State-wise View → pick State → Line of Business = «Offices (Life)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Offices (Life)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1218,6 +1488,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Offices by Region» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Offices by Region</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1245,6 +1525,12 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «the plan / category (Linked, Non-Linked, ULIP, Traditional, Individual/Group)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1272,6 +1558,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Death Claims - Individual» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Micro-Insurance Death Claims - Individual</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1299,6 +1595,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Death Claims - Group» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Micro-Insurance Death Claims - Group</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1326,6 +1632,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Claim Settlement - Individual» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Micro-Insurance Claim Settlement - Individual</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1353,6 +1669,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Claim Settlement - Group» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Micro-Insurance Claim Settlement - Group</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1380,6 +1706,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Grievances (Life)» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Grievances (Life)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1407,6 +1743,16 @@
           <t>Ombudsman Centres → pick Centre → Statement = «Ombudsman Performance (Life)» → Fin Year</t>
         </is>
       </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Ombudsman</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Ombudsman Performance (Life)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1434,6 +1780,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>General (All Segments)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1461,6 +1817,12 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1488,6 +1850,12 @@
           <t>State-wise View → pick State → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1515,6 +1883,16 @@
           <t>Industry-wise View → pick Sector → Line of Business = «Policies Issued» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Policies Issued</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1542,6 +1920,12 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1569,6 +1953,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>General (All Segments)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1596,6 +1990,16 @@
           <t>Industry-wise View → pick Sector → Line of Business = «Investments (AUM)» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Investments (AUM)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1623,6 +2027,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Investments (AUM) by Instrument» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Investments (AUM) by Instrument</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1650,6 +2064,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>General (All Segments)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1677,6 +2101,12 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1704,6 +2134,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Policyholders Account</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1731,6 +2171,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Shareholders Account</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1758,6 +2208,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1785,6 +2245,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Status of Claims» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Status of Claims</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1812,6 +2282,16 @@
           <t>State-wise View → pick State → Line of Business = «Offices (General &amp; Health)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Offices (General &amp; Health)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1839,6 +2319,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Rural / Social Sector Obligations» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Rural / Social Sector Obligations</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1866,6 +2356,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Grievances (General &amp; Health)» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Grievances (General &amp; Health)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1893,6 +2393,16 @@
           <t>Ombudsman Centres → pick Centre → Statement = «Ombudsman Performance (General &amp; Health)» → Fin Year</t>
         </is>
       </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Ombudsman</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Ombudsman Performance (General &amp; Health)</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1920,6 +2430,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Health» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1947,6 +2467,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Personal Accident</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1974,6 +2504,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Travel (Overseas)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2001,6 +2541,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Travel (Domestic)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2028,6 +2578,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Health» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2055,6 +2615,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Personal Accident</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2082,6 +2652,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>Travel (Overseas)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2109,6 +2689,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Travel (Domestic)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2136,6 +2726,16 @@
           <t>Industry-wise View → pick Sector → Line of Business = «Claims Development &amp; Aging» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Claims Development &amp; Aging</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2163,6 +2763,16 @@
           <t>State-wise View → pick State → Line of Business = «Health» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2190,6 +2800,16 @@
           <t>State-wise View → pick State → Line of Business = «Health» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2217,6 +2837,16 @@
           <t>State-wise View → pick State → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Personal Accident</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2244,6 +2874,16 @@
           <t>State-wise View → pick State → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Travel (Overseas)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2271,6 +2911,16 @@
           <t>State-wise View → pick State → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>Travel (Domestic)</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2298,6 +2948,16 @@
           <t>State-wise View → pick State → Line of Business = «Health» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2325,6 +2985,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Health Business by Life Insurers - New» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Health Business by Life Insurers - New</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2352,6 +3022,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Health Business by Life Insurers - Renewal» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Health Business by Life Insurers - Renewal</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2379,6 +3059,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Health Riders on Life Products - New» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Health Riders on Life Products - New</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2406,6 +3096,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Health Riders on Life Products - Renewal» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Health Riders on Life Products - Renewal</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2433,6 +3133,16 @@
           <t>TPA Network → pick TPA → Statement = «Network Hospitals» → Fin Year</t>
         </is>
       </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>TPA</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Network Hospitals</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2460,6 +3170,16 @@
           <t>State-wise View → pick State → Line of Business = «Network Providers» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Network Providers</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2487,6 +3207,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Reinsurance Premium Schedule» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>Reinsurance Premium Schedule</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2514,6 +3244,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Segment-wise Reinsurance Premium Accepted» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>Segment-wise Reinsurance Premium Accepted</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2541,6 +3281,16 @@
           <t>Industry-wise View → pick Sector → Line of Business = «Net Retention (Per cent)» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>Net Retention (Per cent)</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2568,6 +3318,12 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -2595,6 +3351,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Reinsurance» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>Reinsurance</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -2622,6 +3388,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Reinsurance» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>Reinsurance</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -2649,6 +3425,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Reinsurance» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>Reinsurance</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -2676,6 +3462,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>Policyholders Account</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -2703,6 +3499,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>Shareholders Account</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -2730,6 +3536,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>Balance Sheet</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -2757,6 +3573,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -2784,6 +3610,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -2811,6 +3647,16 @@
           <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -2838,6 +3684,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Avg Individual Policies Sold per Agent» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Avg Individual Policies Sold per Agent</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -2865,6 +3721,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Avg New Business Premium per Agent» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Avg New Business Premium per Agent</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -2892,6 +3758,16 @@
           <t>Statements &amp; Reports → pick Insurer → Statement = «Avg Premium per Policy» → Fin Year → Quarter</t>
         </is>
       </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Avg Premium per Policy</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -2919,6 +3795,16 @@
           <t>State-wise View → pick State → Line of Business = «Individual Agents (Life)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Individual Agents (Life)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -2946,6 +3832,16 @@
           <t>State-wise View → pick State → Line of Business = «All Lines» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>All Lines</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -2973,6 +3869,16 @@
           <t>State-wise View → pick State → Line of Business = «All Lines» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>All Lines</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3000,6 +3906,16 @@
           <t>Channel-wise View → pick Channel → Line of Business = «Life - Individual New Business» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Life - Individual New Business</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3027,6 +3943,16 @@
           <t>Channel-wise View → pick Channel → Line of Business = «Life - Group New Business» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Life - Group New Business</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3054,6 +3980,12 @@
           <t>Channel-wise View → pick Channel → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3081,6 +4013,16 @@
           <t>Channel-wise View → pick Channel → Line of Business = «Health» → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -3108,6 +4050,12 @@
           <t>Industry-wise View → pick Sector (Life / General / Indian (All)) → Line of Business → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3135,6 +4083,12 @@
           <t>Country-wise View → pick Country → Line of Business → Metric → Fin Year</t>
         </is>
       </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix Table 4 collision (drop it) + one-click "Open" from access guide
- Table 4 (segment-wise life premium) collided with the summary "Life" LOB and
  is a messy historical breakdown (Linked/Non-Linked × par × premium-type with
  derived Grand Total/Percentage columns + a redundant combined section). Dropped
  — the same linked/non-linked premium is clean per-insurer in Table 12. Also
  taught convert_industry_3col to keep the section prefix (kept for reuse).
- Access guide carries structured Dimension/Pick columns; the in-app guide's
  "Open" button switches to the right view and pre-selects the line of business,
  then opens the filter modal to pick the entity.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/knowledge_base/IRIS_Handbook_Access_Guide.xlsx
+++ b/knowledge_base/IRIS_Handbook_Access_Guide.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -557,30 +557,34 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>TABLE 4: SEGMENT-WISE TOTAL PREMIUM OF LIFE INSURERS</t>
+          <t>TABLE 5: STATE WISE INDIVIDUAL NEW BUSINESS (LIFE) UNDERWRITTEN</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>State-wise</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Life» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Life</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -590,12 +594,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>TABLE 5: STATE WISE INDIVIDUAL NEW BUSINESS (LIFE) UNDERWRITTEN</t>
+          <t>TABLE 6: STATE-WISE INSURER-WISE INDIVIDUAL NEW BUSINESS (LIFE) UNDERWRITTEN (2024-25)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -605,7 +609,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Life» → Class of Biz → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Individual New Business (Life)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -615,7 +619,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Individual New Business (Life)</t>
         </is>
       </c>
     </row>
@@ -627,12 +631,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>TABLE 6: STATE-WISE INSURER-WISE INDIVIDUAL NEW BUSINESS (LIFE) UNDERWRITTEN (2024-25)</t>
+          <t>TABLE 7: STATE WISE GROUP NEW BUSINESS (LIFE) UNDERWRITTEN</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -642,7 +646,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Individual New Business (Life)» → Class of Biz → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Life» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -652,7 +656,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Individual New Business (Life)</t>
+          <t>Life</t>
         </is>
       </c>
     </row>
@@ -664,12 +668,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TABLE 7: STATE WISE GROUP NEW BUSINESS (LIFE) UNDERWRITTEN</t>
+          <t>TABLE 8: STATE WISE INSURER WISE GROUP NEW BUSINESS (LIFE) UNDERWRITTEN</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -679,7 +683,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Life» → Class of Biz → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Group New Business (Life)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -689,7 +693,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Group New Business (Life)</t>
         </is>
       </c>
     </row>
@@ -701,32 +705,32 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>TABLE 8: STATE WISE INSURER WISE GROUP NEW BUSINESS (LIFE) UNDERWRITTEN</t>
+          <t>TABLE 9: NUMBER OF INDIVIDUAL NEW POLICIES ISSUED (LIFE)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>State-wise</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Group New Business (Life)» → Class of Biz → Metric → Fin Year</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Insurer</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Group New Business (Life)</t>
+          <t>Life</t>
         </is>
       </c>
     </row>
@@ -738,32 +742,32 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TABLE 9: NUMBER OF INDIVIDUAL NEW POLICIES ISSUED (LIFE)</t>
+          <t>Table 10: Individual Business inforce (Number of Policies in '000s)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «In-Force Policies» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>In-Force Policies</t>
         </is>
       </c>
     </row>
@@ -775,12 +779,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Table 10: Individual Business inforce (Number of Policies in '000s)</t>
+          <t>Table 11: Individual Business inforce (Sum Assured in ₹Crores)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -790,7 +794,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «In-Force Policies» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «In-Force Sum Assured» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -800,7 +804,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>In-Force Policies</t>
+          <t>In-Force Sum Assured</t>
         </is>
       </c>
     </row>
@@ -812,34 +816,30 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Table 11: Individual Business inforce (Sum Assured in ₹Crores)</t>
+          <t>TABLE 12: LINKED AND NON-LINKED PREMIUM OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «In-Force Sum Assured» → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «the plan / category (Linked, Non-Linked, ULIP, Traditional, Individual/Group)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>In-Force Sum Assured</t>
-        </is>
-      </c>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>TABLE 12: LINKED AND NON-LINKED PREMIUM OF LIFE INSURERS</t>
+          <t>TABLE 13: LINKED AND NON-LINKED COMMISSION OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -882,30 +882,34 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>TABLE 13: LINKED AND NON-LINKED COMMISSION OF LIFE INSURERS</t>
+          <t>TABLE 14: INDIVIDUAL DEATH CLAIMS OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Industry-wise</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «the plan / category (Linked, Non-Linked, ULIP, Traditional, Individual/Group)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Industry-wise View → pick Sector → Line of Business = «Individual Death Claims» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr"/>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Individual Death Claims</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -915,27 +919,27 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>TABLE 14: INDIVIDUAL DEATH CLAIMS OF LIFE INSURERS</t>
+          <t>TABLE 15: INDIVIDUAL DEATH CLAIMS OF LIFE INSURERS - INSURER-WISE</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector → Line of Business = «Individual Death Claims» → Metric → Fin Year</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Individual Death Claims» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -952,32 +956,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>TABLE 15: INDIVIDUAL DEATH CLAIMS OF LIFE INSURERS - INSURER-WISE</t>
+          <t>TABLE 16: GROUP DEATH CLAIMS OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Industry-wise</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Individual Death Claims» → Fin Year → Quarter</t>
+          <t>Industry-wise View → pick Sector → Line of Business = «Group Death Claims» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Individual Death Claims</t>
+          <t>Group Death Claims</t>
         </is>
       </c>
     </row>
@@ -989,27 +993,27 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>TABLE 16: GROUP DEATH CLAIMS OF LIFE INSURERS</t>
+          <t>TABLE 17: GROUP DEATH CLAIMS OF LIFE INSURERS - INSURER-WISE</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector → Line of Business = «Group Death Claims» → Metric → Fin Year</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Group Death Claims» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1026,12 +1030,12 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>TABLE 17: GROUP DEATH CLAIMS OF LIFE INSURERS - INSURER-WISE</t>
+          <t>TABLE 18: DURATION WISE SETTLEMENT OF DEATH CLAIMS - INDIVIDUAL CATEGORY</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1041,7 +1045,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Group Death Claims» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Death Claim Settlement Duration - Individual» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1051,7 +1055,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Group Death Claims</t>
+          <t>Death Claim Settlement Duration - Individual</t>
         </is>
       </c>
     </row>
@@ -1063,12 +1067,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>TABLE 18: DURATION WISE SETTLEMENT OF DEATH CLAIMS - INDIVIDUAL CATEGORY</t>
+          <t>TABLE 19: DURATION WISE SETTLEMENT OF DEATH CLAIMS - GROUP CATEGORY</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1078,7 +1082,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Death Claim Settlement Duration - Individual» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Death Claim Settlement Duration - Group» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1088,7 +1092,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Death Claim Settlement Duration - Individual</t>
+          <t>Death Claim Settlement Duration - Group</t>
         </is>
       </c>
     </row>
@@ -1100,32 +1104,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>TABLE 19: DURATION WISE SETTLEMENT OF DEATH CLAIMS - GROUP CATEGORY</t>
+          <t>TABLE 20: ASSETS UNDER MANAGEMENT (INVESTMENTS) OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Industry-wise</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Death Claim Settlement Duration - Group» → Fin Year → Quarter</t>
+          <t>Industry-wise View → pick Sector → Line of Business = «Investments (AUM)» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Death Claim Settlement Duration - Group</t>
+          <t>Investments (AUM)</t>
         </is>
       </c>
     </row>
@@ -1137,32 +1141,32 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>TABLE 20: ASSETS UNDER MANAGEMENT (INVESTMENTS) OF LIFE INSURERS</t>
+          <t>TABLE 22: EQUITY SHARE CAPITAL OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector → Line of Business = «Investments (AUM)» → Metric → Fin Year</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Insurer</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Investments (AUM)</t>
+          <t>Life</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1178,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>TABLE 22: EQUITY SHARE CAPITAL OF LIFE INSURERS</t>
+          <t>Table 23: Solvency Ratio of Life Insurers</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1211,32 +1215,32 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Table 23: Solvency Ratio of Life Insurers</t>
+          <t>TABLE 24: POLICYHOLDERS ACCOUNT OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Policyholders Account</t>
         </is>
       </c>
     </row>
@@ -1248,12 +1252,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>TABLE 24: POLICYHOLDERS ACCOUNT OF LIFE INSURERS</t>
+          <t>TABLE 25: SHAREHOLDERS ACCOUNT OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1263,7 +1267,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1273,7 +1277,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Policyholders Account</t>
+          <t>Shareholders Account</t>
         </is>
       </c>
     </row>
@@ -1285,12 +1289,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>TABLE 25: SHAREHOLDERS ACCOUNT OF LIFE INSURERS</t>
+          <t>TABLE 26: BALANCE SHEET OF LIFE INSURERS (As on 31st March)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1300,7 +1304,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1310,7 +1314,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Shareholders Account</t>
+          <t>Balance Sheet</t>
         </is>
       </c>
     </row>
@@ -1322,12 +1326,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>TABLE 26: BALANCE SHEET OF LIFE INSURERS (As on 31st March)</t>
+          <t>TABLE 27: DETAILS OF FORFEITURE/LAPSED POLICIES IN RESPECT OF INDIVIDUAL NON-LINKED BUSINESS (EXCLUDING VIP) (WITHIN INDIA)</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1337,7 +1341,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Lapsed / Forfeited Policies (Non-Linked)» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1347,7 +1351,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Balance Sheet</t>
+          <t>Lapsed / Forfeited Policies (Non-Linked)</t>
         </is>
       </c>
     </row>
@@ -1359,12 +1363,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>TABLE 27: DETAILS OF FORFEITURE/LAPSED POLICIES IN RESPECT OF INDIVIDUAL NON-LINKED BUSINESS (EXCLUDING VIP) (WITHIN INDIA)</t>
+          <t>TABLE 28: PERSISTENCY OF LIFE INSURANCE POLICIES (BASED ON NUMBER OF POLICIES)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1374,7 +1378,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Lapsed / Forfeited Policies (Non-Linked)» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Persistency» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1384,7 +1388,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Lapsed / Forfeited Policies (Non-Linked)</t>
+          <t>Persistency</t>
         </is>
       </c>
     </row>
@@ -1396,32 +1400,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>TABLE 28: PERSISTENCY OF LIFE INSURANCE POLICIES (BASED ON NUMBER OF POLICIES)</t>
+          <t>TABLE 29: STATE-WISE DISTRIBUTION OF OFFICES OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>State-wise</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Persistency» → Fin Year → Quarter</t>
+          <t>State-wise View → pick State → Line of Business = «Offices (Life)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>State</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Persistency</t>
+          <t>Offices (Life)</t>
         </is>
       </c>
     </row>
@@ -1433,32 +1437,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>TABLE 29: STATE-WISE DISTRIBUTION OF OFFICES OF LIFE INSURERS</t>
+          <t>TABLE 30: REGION-WISE DISTRIBUTION OF OFFICES OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>State-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Offices (Life)» → Class of Biz → Metric → Fin Year</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Offices by Region» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Offices (Life)</t>
+          <t>Offices by Region</t>
         </is>
       </c>
     </row>
@@ -1470,34 +1474,30 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>TABLE 30: REGION-WISE DISTRIBUTION OF OFFICES OF LIFE INSURERS</t>
+          <t>TABLE 31: NEW BUSINESS UNDER MICRO-INSURANCE PORTFOLIO -LIFE INSURERS</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Offices by Region» → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «the plan / category (Linked, Non-Linked, ULIP, Traditional, Individual/Group)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Offices by Region</t>
-        </is>
-      </c>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1507,30 +1507,34 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>TABLE 31: NEW BUSINESS UNDER MICRO-INSURANCE PORTFOLIO -LIFE INSURERS</t>
+          <t>TABLE 32: DEATH CLAIMS UNDER MICRO- INSURANCE PORTFOLIO - INDIVIDUAL CATEGORY</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «the plan / category (Linked, Non-Linked, ULIP, Traditional, Individual/Group)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Death Claims - Individual» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr"/>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Micro-Insurance Death Claims - Individual</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1540,12 +1544,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>TABLE 32: DEATH CLAIMS UNDER MICRO- INSURANCE PORTFOLIO - INDIVIDUAL CATEGORY</t>
+          <t>TABLE 33: DEATH CLAIMS UNDER MICRO- INSURANCE PORTFOLIO - GROUP CATEGORY</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1555,7 +1559,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Death Claims - Individual» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Death Claims - Group» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1565,7 +1569,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Micro-Insurance Death Claims - Individual</t>
+          <t>Micro-Insurance Death Claims - Group</t>
         </is>
       </c>
     </row>
@@ -1577,12 +1581,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>34</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>TABLE 33: DEATH CLAIMS UNDER MICRO- INSURANCE PORTFOLIO - GROUP CATEGORY</t>
+          <t>TABLE 34: DURATION-WISE SETTLEMENT OF CLAIMS-MICRO INSURANCE - INDIVIDUAL CATEGORY</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1592,7 +1596,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Death Claims - Group» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Claim Settlement - Individual» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1602,7 +1606,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Micro-Insurance Death Claims - Group</t>
+          <t>Micro-Insurance Claim Settlement - Individual</t>
         </is>
       </c>
     </row>
@@ -1614,12 +1618,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>TABLE 34: DURATION-WISE SETTLEMENT OF CLAIMS-MICRO INSURANCE - INDIVIDUAL CATEGORY</t>
+          <t>TABLE 35: DURATION-WISE SETTLEMENT OF CLAIMS-MICRO INSURANCE - GROUP CATEGORY</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1629,7 +1633,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Claim Settlement - Individual» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Claim Settlement - Group» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1639,7 +1643,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Micro-Insurance Claim Settlement - Individual</t>
+          <t>Micro-Insurance Claim Settlement - Group</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1655,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>TABLE 35: DURATION-WISE SETTLEMENT OF CLAIMS-MICRO INSURANCE - GROUP CATEGORY</t>
+          <t>TABLE 37: STATUS OF GRIEVANCES WITH LIFE INSURERS</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1666,7 +1670,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Micro-Insurance Claim Settlement - Group» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Grievances (Life)» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1676,7 +1680,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Micro-Insurance Claim Settlement - Group</t>
+          <t>Grievances (Life)</t>
         </is>
       </c>
     </row>
@@ -1688,69 +1692,69 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>38</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>TABLE 37: STATUS OF GRIEVANCES WITH LIFE INSURERS</t>
+          <t>TABLE 38: PERFORMANCE OF OMBUDSMEN AT DIFFERENT CENTRES-LIFE INSURANCE</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Ombudsman-wise</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Grievances (Life)» → Fin Year → Quarter</t>
+          <t>Ombudsman Centres → pick Centre → Statement = «Ombudsman Performance (Life)» → Fin Year</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Ombudsman</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Grievances (Life)</t>
+          <t>Ombudsman Performance (Life)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Part I</t>
+          <t>Part II</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>40</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>TABLE 38: PERFORMANCE OF OMBUDSMEN AT DIFFERENT CENTRES-LIFE INSURANCE</t>
+          <t>TABLE 40 GROSS DIRECT PREMIUM OF GENERAL AND HEALTH INSURERS (WITHIN AND OUTSIDE INDIA)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Ombudsman-wise</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Ombudsman Centres → pick Centre → Statement = «Ombudsman Performance (Life)» → Fin Year</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Ombudsman</t>
+          <t>Insurer</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Ombudsman Performance (Life)</t>
+          <t>General (All Segments)</t>
         </is>
       </c>
     </row>
@@ -1762,12 +1766,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>41</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>TABLE 40 GROSS DIRECT PREMIUM OF GENERAL AND HEALTH INSURERS (WITHIN AND OUTSIDE INDIA)</t>
+          <t>TABLE 41: SEGMENT-WISE GROSS DIRECT PREMIUM OF GENERAL AND HEALTH INSURERS (WITHIN INDIA)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1777,7 +1781,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1785,11 +1789,7 @@
           <t>Insurer</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>General (All Segments)</t>
-        </is>
-      </c>
+      <c r="G37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1799,27 +1799,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>42</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>TABLE 41: SEGMENT-WISE GROSS DIRECT PREMIUM OF GENERAL AND HEALTH INSURERS (WITHIN INDIA)</t>
+          <t>TABLE 42: STATE-WISE GROSS DIRECT PREMIUM-GENERAL INSURANCE</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>State-wise</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>State-wise View → pick State → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
+          <t>State</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
@@ -1832,30 +1832,34 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>43</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>TABLE 42: STATE-WISE GROSS DIRECT PREMIUM-GENERAL INSURANCE</t>
+          <t>STATEMENT 43: NUMBER OF POLICIES ISSUED BY GENERAL INSURERS</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>State-wise</t>
+          <t>Industry-wise</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year</t>
+          <t>Industry-wise View → pick Sector → Line of Business = «Policies Issued» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr"/>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Policies Issued</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1865,34 +1869,30 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>44</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>STATEMENT 43: NUMBER OF POLICIES ISSUED BY GENERAL INSURERS</t>
+          <t>TABLE 44: NET PREMIUM EARNED, INCURRED CLAIMS AND INCURRED CLAIMS RATIO OF GENERAL AND HEALTH INSURERS (WITHIN INDIA)</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector → Line of Business = «Policies Issued» → Metric → Fin Year</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Policies Issued</t>
-        </is>
-      </c>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1902,12 +1902,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>45</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>TABLE 44: NET PREMIUM EARNED, INCURRED CLAIMS AND INCURRED CLAIMS RATIO OF GENERAL AND HEALTH INSURERS (WITHIN INDIA)</t>
+          <t>TABLE 45: UNDERWRITING EXPERIENCE OF GENERAL AND HEALTH INSURERS</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1925,7 +1925,11 @@
           <t>Insurer</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>General (All Segments)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1935,32 +1939,32 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>TABLE 45: UNDERWRITING EXPERIENCE OF GENERAL AND HEALTH INSURERS</t>
+          <t>TABLE 46: ASSETS UNDER MANAGEMENT (INVESTMENTS) OF GENERAL, HELATH AND REINSURANCE COMPANIES</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Industry-wise</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Industry-wise View → pick Sector → Line of Business = «Investments (AUM)» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>General (All Segments)</t>
+          <t>Investments (AUM)</t>
         </is>
       </c>
     </row>
@@ -1972,32 +1976,32 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>47</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>TABLE 46: ASSETS UNDER MANAGEMENT (INVESTMENTS) OF GENERAL, HELATH AND REINSURANCE COMPANIES</t>
+          <t>TABLE 47: INVESTMENTS (ASSETS UNDER MANAGEMENT) OF GENERAL, HEALTH AND REINSURANCE COMPANIES - INSURER WISE</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector → Line of Business = «Investments (AUM)» → Metric → Fin Year</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Investments (AUM) by Instrument» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Investments (AUM)</t>
+          <t>Investments (AUM) by Instrument</t>
         </is>
       </c>
     </row>
@@ -2009,32 +2013,32 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>TABLE 47: INVESTMENTS (ASSETS UNDER MANAGEMENT) OF GENERAL, HEALTH AND REINSURANCE COMPANIES - INSURER WISE</t>
+          <t>TABLE 48: EQUITY SHARE CAPITAL OF GENERAL AND HEALTH INSURERS</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Investments (AUM) by Instrument» → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Insurer</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Investments (AUM) by Instrument</t>
+          <t>General (All Segments)</t>
         </is>
       </c>
     </row>
@@ -2046,12 +2050,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>TABLE 48: EQUITY SHARE CAPITAL OF GENERAL AND HEALTH INSURERS</t>
+          <t>TABLE 49: SOLVENCY RATIO OF GENERAL, HEALTH AND REINSURANCE COMPANIES</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -2061,7 +2065,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «General» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -2069,11 +2073,7 @@
           <t>Insurer</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>General (All Segments)</t>
-        </is>
-      </c>
+      <c r="G45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2083,30 +2083,34 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>50</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>TABLE 49: SOLVENCY RATIO OF GENERAL, HEALTH AND REINSURANCE COMPANIES</t>
+          <t>TABLE 50: POLICYHOLDERS ACCOUNT OF GENERAL AND HEALTH INSURERS</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Policyholders Account</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2116,12 +2120,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>51</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>TABLE 50: POLICYHOLDERS ACCOUNT OF GENERAL AND HEALTH INSURERS</t>
+          <t>TABLE 51: SHAREHOLDERS ACCOUNT OF GENERAL AND HEALTH INSURERS</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2131,7 +2135,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2141,7 +2145,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Policyholders Account</t>
+          <t>Shareholders Account</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2157,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>52</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>TABLE 51: SHAREHOLDERS ACCOUNT OF GENERAL AND HEALTH INSURERS</t>
+          <t>TABLE 52: BALANCE SHEET OF GENERAL AND HEALTH INSURERS (AS AT 31ST MARCH)</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -2168,7 +2172,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2178,7 +2182,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Shareholders Account</t>
+          <t>Balance Sheet</t>
         </is>
       </c>
     </row>
@@ -2190,12 +2194,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>53</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>TABLE 52: BALANCE SHEET OF GENERAL AND HEALTH INSURERS (AS AT 31ST MARCH)</t>
+          <t>TABLE 53: STATUS OF CLAIMS OF GENERAL AND HEALTH INSURERS</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -2205,7 +2209,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Status of Claims» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -2215,7 +2219,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Balance Sheet</t>
+          <t>Status of Claims</t>
         </is>
       </c>
     </row>
@@ -2227,32 +2231,32 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>54</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>TABLE 53: STATUS OF CLAIMS OF GENERAL AND HEALTH INSURERS</t>
+          <t>TABLE 54: STATE-WISE DISTRIBUTION OF OFFICES OF GENERAL AND HEALTH INSURERS</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>State-wise</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Status of Claims» → Fin Year → Quarter</t>
+          <t>State-wise View → pick State → Line of Business = «Offices (General &amp; Health)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>State</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Status of Claims</t>
+          <t>Offices (General &amp; Health)</t>
         </is>
       </c>
     </row>
@@ -2264,32 +2268,32 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>55</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>TABLE 54: STATE-WISE DISTRIBUTION OF OFFICES OF GENERAL AND HEALTH INSURERS</t>
+          <t>TABLE 55: RURAL AND SOCIAL SECTOR OBLIGATIONS OF GENERAL AND HEALTH INSURERS</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>State-wise</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Offices (General &amp; Health)» → Class of Biz → Metric → Fin Year</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Rural / Social Sector Obligations» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Insurer</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Offices (General &amp; Health)</t>
+          <t>Rural / Social Sector Obligations</t>
         </is>
       </c>
     </row>
@@ -2301,32 +2305,32 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>56</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>TABLE 55: RURAL AND SOCIAL SECTOR OBLIGATIONS OF GENERAL AND HEALTH INSURERS</t>
+          <t>TABLE 56: STATUS OF GRIEVANCES WITH GENERAL AND HEALTH INSURER</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Rural / Social Sector Obligations» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Grievances (General &amp; Health)» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Rural / Social Sector Obligations</t>
+          <t>Grievances (General &amp; Health)</t>
         </is>
       </c>
     </row>
@@ -2338,69 +2342,69 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>57</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>TABLE 56: STATUS OF GRIEVANCES WITH GENERAL AND HEALTH INSURER</t>
+          <t>TABLE 57: PERFORMANCE OF OMBUDSMEN AT DIFFERENT CENTRES - GENERAL AND HEALTH INSURANCE</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Ombudsman-wise</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Grievances (General &amp; Health)» → Fin Year → Quarter</t>
+          <t>Ombudsman Centres → pick Centre → Statement = «Ombudsman Performance (General &amp; Health)» → Fin Year</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Ombudsman</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Grievances (General &amp; Health)</t>
+          <t>Ombudsman Performance (General &amp; Health)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Part II</t>
+          <t>Part III</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>58</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>TABLE 57: PERFORMANCE OF OMBUDSMEN AT DIFFERENT CENTRES - GENERAL AND HEALTH INSURANCE</t>
+          <t>TABLE 58: HEALTH INSURANCE (EXCLUDING PERSONAL ACCIDENT AND TRAVEL) - NUMBER OF POLICIES, NUMBER OF PERSONS COVERED AND GROSS PREMIUM</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Ombudsman-wise</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Ombudsman Centres → pick Centre → Statement = «Ombudsman Performance (General &amp; Health)» → Fin Year</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Health» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Ombudsman</t>
+          <t>Insurer</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Ombudsman Performance (General &amp; Health)</t>
+          <t>Health</t>
         </is>
       </c>
     </row>
@@ -2412,12 +2416,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>59</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>TABLE 58: HEALTH INSURANCE (EXCLUDING PERSONAL ACCIDENT AND TRAVEL) - NUMBER OF POLICIES, NUMBER OF PERSONS COVERED AND GROSS PREMIUM</t>
+          <t>TABLE 59: PERSONAL ACCIDENT INSURANCE - NUMBER OF POLICIES, NUMBER OF PERSONS COVERED AND GROSS PREMIUM</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -2427,7 +2431,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Health» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2437,7 +2441,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Personal Accident</t>
         </is>
       </c>
     </row>
@@ -2449,12 +2453,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>TABLE 59: PERSONAL ACCIDENT INSURANCE - NUMBER OF POLICIES, NUMBER OF PERSONS COVERED AND GROSS PREMIUM</t>
+          <t>TABLE 60: OVERSEAS TRAVEL INSURANCE - NUMBER OF POLICIES, NUMBER OF PERSONS COVERED AND GROSS PREMIUM</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -2464,7 +2468,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2474,7 +2478,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Personal Accident</t>
+          <t>Travel (Overseas)</t>
         </is>
       </c>
     </row>
@@ -2486,12 +2490,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>61</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>TABLE 60: OVERSEAS TRAVEL INSURANCE - NUMBER OF POLICIES, NUMBER OF PERSONS COVERED AND GROSS PREMIUM</t>
+          <t>TABLE 61: DOMESTIC TRAVEL INSURANCE - NUMBER OF POLICIES, NUMBER OF PERSONS COVERED AND GROSS PREMIUM</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -2501,7 +2505,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2511,7 +2515,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Travel (Overseas)</t>
+          <t>Travel (Domestic)</t>
         </is>
       </c>
     </row>
@@ -2523,12 +2527,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>TABLE 61: DOMESTIC TRAVEL INSURANCE - NUMBER OF POLICIES, NUMBER OF PERSONS COVERED AND GROSS PREMIUM</t>
+          <t>TABLE 62: HEALTH INSURANCE (EXCLUDING PERSONAL ACCIDENT AND TRAVEL) - NET EARNED PREMIUM, INCURRED CLAIMS AND INCURRED CLAIMS RATIO</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -2538,7 +2542,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Health» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2548,7 +2552,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Travel (Domestic)</t>
+          <t>Health</t>
         </is>
       </c>
     </row>
@@ -2560,12 +2564,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>63</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>TABLE 62: HEALTH INSURANCE (EXCLUDING PERSONAL ACCIDENT AND TRAVEL) - NET EARNED PREMIUM, INCURRED CLAIMS AND INCURRED CLAIMS RATIO</t>
+          <t>TABLE 63: PERSONAL ACCIDENT INSURANCE - NET EARNED PREMIUM, NET CLAIMS INCURRED AND INCURRED CLAIMS RATIO</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -2575,7 +2579,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Health» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2585,7 +2589,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Personal Accident</t>
         </is>
       </c>
     </row>
@@ -2597,12 +2601,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>64</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>TABLE 63: PERSONAL ACCIDENT INSURANCE - NET EARNED PREMIUM, NET CLAIMS INCURRED AND INCURRED CLAIMS RATIO</t>
+          <t>TABLE 64: OVERSEAS TRAVEL INSURANCE -NET EARNED PREMIUM, NET CLAIMS INCURRED AND INCURRED CLAIMS RATIO</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -2612,7 +2616,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2622,7 +2626,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Personal Accident</t>
+          <t>Travel (Overseas)</t>
         </is>
       </c>
     </row>
@@ -2634,12 +2638,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>65</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>TABLE 64: OVERSEAS TRAVEL INSURANCE -NET EARNED PREMIUM, NET CLAIMS INCURRED AND INCURRED CLAIMS RATIO</t>
+          <t>TABLE 65: DOMESTIC TRAVEL INSURANCE - NET EARNED PREMIUM, NET CLAIMS INCURRED AND INCURRED CLAIMS RATIO</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -2649,7 +2653,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2659,7 +2663,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Travel (Overseas)</t>
+          <t>Travel (Domestic)</t>
         </is>
       </c>
     </row>
@@ -2671,32 +2675,32 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>TABLE 65: DOMESTIC TRAVEL INSURANCE - NET EARNED PREMIUM, NET CLAIMS INCURRED AND INCURRED CLAIMS RATIO</t>
+          <t>TABLE 66: DETAILS OF CLAIMS DEVELOPMENT AND AGING - HEALTH INSURANCE BUSINESS (EXCLUDING TRAVEL AND PERSONAL ACCIDENT)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Industry-wise</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Industry-wise View → pick Sector → Line of Business = «Claims Development &amp; Aging» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Travel (Domestic)</t>
+          <t>Claims Development &amp; Aging</t>
         </is>
       </c>
     </row>
@@ -2708,32 +2712,32 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>67</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>TABLE 66: DETAILS OF CLAIMS DEVELOPMENT AND AGING - HEALTH INSURANCE BUSINESS (EXCLUDING TRAVEL AND PERSONAL ACCIDENT)</t>
+          <t>TABLE 67: STATE-WISE HEALTH INSURANCE BUSINESS (EXCLUDING TRAVEL AND PERSONAL ACCIDENT BUSINESS)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>State-wise</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector → Line of Business = «Claims Development &amp; Aging» → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Health» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>State</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Claims Development &amp; Aging</t>
+          <t>Health</t>
         </is>
       </c>
     </row>
@@ -2745,12 +2749,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>68</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>TABLE 67: STATE-WISE HEALTH INSURANCE BUSINESS (EXCLUDING TRAVEL AND PERSONAL ACCIDENT BUSINESS)</t>
+          <t>TABLE 68: STATE-WISE INDIVIDUAL HEALTH INSURANCE BUSINESS (EXCL. PA &amp; TRAVEL BUSINESS)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -2782,12 +2786,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>TABLE 68: STATE-WISE INDIVIDUAL HEALTH INSURANCE BUSINESS (EXCL. PA &amp; TRAVEL BUSINESS)</t>
+          <t>TABLE 69: STATE WISE PERSONAL ACCIDENT INSURANCE BUSINESSS (Exclusive of business from IRCTC &amp; PMJDY Schemes)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -2797,7 +2801,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Health» → Class of Biz → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2807,7 +2811,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Personal Accident</t>
         </is>
       </c>
     </row>
@@ -2819,12 +2823,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>TABLE 69: STATE WISE PERSONAL ACCIDENT INSURANCE BUSINESSS (Exclusive of business from IRCTC &amp; PMJDY Schemes)</t>
+          <t>TABLE 70: STATE WISE OVERSEAS TRAVEL INSURANCE BUSINESSS</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -2834,7 +2838,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Personal Accident» → Class of Biz → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -2844,7 +2848,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Personal Accident</t>
+          <t>Travel (Overseas)</t>
         </is>
       </c>
     </row>
@@ -2856,12 +2860,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>71</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>TABLE 70: STATE WISE OVERSEAS TRAVEL INSURANCE BUSINESSS</t>
+          <t>TABLE 71: STATE WISE DOMESTIC TRAVEL INSURANCE BUSINESSS</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -2871,7 +2875,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Travel (Overseas)» → Class of Biz → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -2881,7 +2885,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Travel (Overseas)</t>
+          <t>Travel (Domestic)</t>
         </is>
       </c>
     </row>
@@ -2893,12 +2897,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>72</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>TABLE 71: STATE WISE DOMESTIC TRAVEL INSURANCE BUSINESSS</t>
+          <t>TABLE 72: STATE-WISE CLAIM SETTLEMENT UNDER HEALTH INSURANCE BUSINESS</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -2908,7 +2912,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Travel (Domestic)» → Class of Biz → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Health» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -2918,7 +2922,7 @@
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Travel (Domestic)</t>
+          <t>Health</t>
         </is>
       </c>
     </row>
@@ -2930,32 +2934,32 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>73</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>TABLE 72: STATE-WISE CLAIM SETTLEMENT UNDER HEALTH INSURANCE BUSINESS</t>
+          <t>TABLE 73: HEALTH INSURANCE BUSINESS IN RESPECT OF HEALTH PRODUCTS OFFERED BY LIFE INSURERS - NEW BUSINESS</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>State-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Health» → Class of Biz → Metric → Fin Year</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Health Business by Life Insurers - New» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Health Business by Life Insurers - New</t>
         </is>
       </c>
     </row>
@@ -2967,12 +2971,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>74</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>TABLE 73: HEALTH INSURANCE BUSINESS IN RESPECT OF HEALTH PRODUCTS OFFERED BY LIFE INSURERS - NEW BUSINESS</t>
+          <t>TABLE 74: HEALTH INSURANCE BUSINESS IN RESPECT OF HEALTH PRODUCTS OFFERED BY LIFE INSURERS - RENEWAL BUSINESS</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -2982,7 +2986,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Health Business by Life Insurers - New» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Health Business by Life Insurers - Renewal» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2992,7 +2996,7 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Health Business by Life Insurers - New</t>
+          <t>Health Business by Life Insurers - Renewal</t>
         </is>
       </c>
     </row>
@@ -3004,12 +3008,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>75</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>TABLE 74: HEALTH INSURANCE BUSINESS IN RESPECT OF HEALTH PRODUCTS OFFERED BY LIFE INSURERS - RENEWAL BUSINESS</t>
+          <t>TABLE 75: HEALTH INSURANCE BUSINESS IN RESPECT OF RIDERS ATTACHED TO THE LIFE INSURANCE PRODUCTS OFFERED BY LIFE INSURERS -NEW BUSINESS</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -3019,7 +3023,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Health Business by Life Insurers - Renewal» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Health Riders on Life Products - New» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -3029,7 +3033,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Health Business by Life Insurers - Renewal</t>
+          <t>Health Riders on Life Products - New</t>
         </is>
       </c>
     </row>
@@ -3041,12 +3045,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>76</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>TABLE 75: HEALTH INSURANCE BUSINESS IN RESPECT OF RIDERS ATTACHED TO THE LIFE INSURANCE PRODUCTS OFFERED BY LIFE INSURERS -NEW BUSINESS</t>
+          <t>TABLE 76: HEALTH INSURANCE BUSINESS IN RESPECT OF RIDERS ATTACHED TO LIFE INSURANCE PRODUCTS OFFERED BY LIFE INSURANCE COMPANIES - RENEWAL BUSINESS</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -3056,7 +3060,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Health Riders on Life Products - New» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Health Riders on Life Products - Renewal» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -3066,7 +3070,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Health Riders on Life Products - New</t>
+          <t>Health Riders on Life Products - Renewal</t>
         </is>
       </c>
     </row>
@@ -3078,32 +3082,32 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>77</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>TABLE 76: HEALTH INSURANCE BUSINESS IN RESPECT OF RIDERS ATTACHED TO LIFE INSURANCE PRODUCTS OFFERED BY LIFE INSURANCE COMPANIES - RENEWAL BUSINESS</t>
+          <t>TABLE 77: NETWORK HOSPITAL ENROLLED BY TPAs</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>TPA-wise</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Health Riders on Life Products - Renewal» → Fin Year → Quarter</t>
+          <t>TPA Network → pick TPA → Statement = «Network Hospitals» → Fin Year</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>TPA</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Health Riders on Life Products - Renewal</t>
+          <t>Network Hospitals</t>
         </is>
       </c>
     </row>
@@ -3115,69 +3119,69 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>TABLE 77: NETWORK HOSPITAL ENROLLED BY TPAs</t>
+          <t>TABLE 80: STATE-WISE DETAILS ON NUMBER OF NETWORK PROVIDERS (2024-25)</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>TPA-wise</t>
+          <t>State-wise</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>TPA Network → pick TPA → Statement = «Network Hospitals» → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «Network Providers» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>TPA</t>
+          <t>State</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Network Hospitals</t>
+          <t>Network Providers</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Part III</t>
+          <t>Part IV</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>78</t>
+          <t>80</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>TABLE 80: STATE-WISE DETAILS ON NUMBER OF NETWORK PROVIDERS (2024-25)</t>
+          <t>TABLE 80: PREMIUM SCHEDULE OF REINSURERS</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>State-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Network Providers» → Class of Biz → Metric → Fin Year</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Reinsurance Premium Schedule» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Network Providers</t>
+          <t>Reinsurance Premium Schedule</t>
         </is>
       </c>
     </row>
@@ -3189,12 +3193,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>81</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>TABLE 80: PREMIUM SCHEDULE OF REINSURERS</t>
+          <t>TABLE 81: SEGMENT-WISE PREMIUM ON REINSURANCE / RETROCESSION ACCEPTED</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -3204,7 +3208,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Reinsurance Premium Schedule» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Segment-wise Reinsurance Premium Accepted» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -3214,7 +3218,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Reinsurance Premium Schedule</t>
+          <t>Segment-wise Reinsurance Premium Accepted</t>
         </is>
       </c>
     </row>
@@ -3226,32 +3230,32 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>82</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>TABLE 81: SEGMENT-WISE PREMIUM ON REINSURANCE / RETROCESSION ACCEPTED</t>
+          <t>Table 82: Net Retention of Non-Life Insurers, Indian Reinsurers and Foreign Reinsurers' Branches in India</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Industry-wise</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Segment-wise Reinsurance Premium Accepted» → Fin Year → Quarter</t>
+          <t>Industry-wise View → pick Sector → Line of Business = «Net Retention (Per cent)» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industry</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Segment-wise Reinsurance Premium Accepted</t>
+          <t>Net Retention (Per cent)</t>
         </is>
       </c>
     </row>
@@ -3263,34 +3267,30 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Table 82: Net Retention of Non-Life Insurers, Indian Reinsurers and Foreign Reinsurers' Branches in India</t>
+          <t>TABLE 83: NET EARNED PREMIUM, INCURRED CLAIMS AND INCURRED CLAIMS RATIO OF REINSURERS</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector → Line of Business = «Net Retention (Per cent)» → Metric → Fin Year</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>Net Retention (Per cent)</t>
-        </is>
-      </c>
+          <t>Insurer</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3300,12 +3300,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>84</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>TABLE 83: NET EARNED PREMIUM, INCURRED CLAIMS AND INCURRED CLAIMS RATIO OF REINSURERS</t>
+          <t>TABLE 84: UNDERWRITING EXPERIENCE OF REINSURERS</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Reinsurance» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -3323,7 +3323,11 @@
           <t>Insurer</t>
         </is>
       </c>
-      <c r="G79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>Reinsurance</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3333,12 +3337,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>85</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>TABLE 84: UNDERWRITING EXPERIENCE OF REINSURERS</t>
+          <t>TABLE 85: EQUITY SHARE CAPITAL OF REINSURERS/ASSIGNED CAPITAL OF BRANCHES OF FOREIGN REINSURERS</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -3370,12 +3374,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>86</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>TABLE 85: EQUITY SHARE CAPITAL OF REINSURERS/ASSIGNED CAPITAL OF BRANCHES OF FOREIGN REINSURERS</t>
+          <t>TABLE 86: SOLVENCY RATIO OF REINSURERS</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -3407,32 +3411,32 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>87</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>TABLE 86: SOLVENCY RATIO OF REINSURERS</t>
+          <t>TABLE 87: POLICYHOLDERS ACCOUNT OF REINSURERS</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Reinsurance» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Reinsurance</t>
+          <t>Policyholders Account</t>
         </is>
       </c>
     </row>
@@ -3444,12 +3448,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>88</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>TABLE 87: POLICYHOLDERS ACCOUNT OF REINSURERS</t>
+          <t>TABLE 88: SHAREHOLDERS ACCOUNT OF REINSURERS</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -3459,7 +3463,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Policyholders Account» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -3469,7 +3473,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Policyholders Account</t>
+          <t>Shareholders Account</t>
         </is>
       </c>
     </row>
@@ -3481,12 +3485,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>89</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>TABLE 88: SHAREHOLDERS ACCOUNT OF REINSURERS</t>
+          <t>TABLE 89: BALANCE SHEET OF REINSURERS</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -3496,7 +3500,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Shareholders Account» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -3506,44 +3510,44 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Shareholders Account</t>
+          <t>Balance Sheet</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Part IV</t>
+          <t>Part V</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>TABLE 89: BALANCE SHEET OF REINSURERS</t>
+          <t>TABLE 90: NUMBER OF INDIVIDUAL AGENTS OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>Insurer-wise</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Balance Sheet» → Fin Year → Quarter</t>
+          <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Insurer</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Balance Sheet</t>
+          <t>Life</t>
         </is>
       </c>
     </row>
@@ -3555,12 +3559,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>91</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>TABLE 90: NUMBER OF INDIVIDUAL AGENTS OF LIFE INSURERS</t>
+          <t>TABLE 91: NUMBER OF CORPORATE AGENTS OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -3592,12 +3596,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>92</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>TABLE 91: NUMBER OF CORPORATE AGENTS OF LIFE INSURERS</t>
+          <t>TABLE 92: NUMBER OF MICRO INSURANCE AGENTS (LIFE) - INSURER-WISE</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -3629,32 +3633,32 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>93</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>TABLE 92: NUMBER OF MICRO INSURANCE AGENTS (LIFE) - INSURER-WISE</t>
+          <t>TABLE 93: AVERAGE NUMBER OF INDIVIDUAL POLICIES SOLD BY INDIVIDUAL AND CORPORATE AGENTS</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise</t>
+          <t>Statements &amp; Reports</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Insurer-wise View → pick Insurer → Line of Business = «Life» → Class of Biz → Metric → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Avg Individual Policies Sold per Agent» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Insurer</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Life</t>
+          <t>Avg Individual Policies Sold per Agent</t>
         </is>
       </c>
     </row>
@@ -3666,12 +3670,12 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>94</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>TABLE 93: AVERAGE NUMBER OF INDIVIDUAL POLICIES SOLD BY INDIVIDUAL AND CORPORATE AGENTS</t>
+          <t>TABLE 94: AVERAGE NEW BUSINESS PREMIUM INCOME PER INDIVIDUAL AND CORPORATE AGENTS</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -3681,7 +3685,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Avg Individual Policies Sold per Agent» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Avg New Business Premium per Agent» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -3691,7 +3695,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Avg Individual Policies Sold per Agent</t>
+          <t>Avg New Business Premium per Agent</t>
         </is>
       </c>
     </row>
@@ -3703,12 +3707,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>95</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>TABLE 94: AVERAGE NEW BUSINESS PREMIUM INCOME PER INDIVIDUAL AND CORPORATE AGENTS</t>
+          <t>TABLE 95: AVERAGE PREMIUM INCOME PER POLICY FOR INDIVIDUAL AND CORPORATE AGENTS</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -3718,7 +3722,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Avg New Business Premium per Agent» → Fin Year → Quarter</t>
+          <t>Statements &amp; Reports → pick Insurer → Statement = «Avg Premium per Policy» → Fin Year → Quarter</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -3728,7 +3732,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Avg New Business Premium per Agent</t>
+          <t>Avg Premium per Policy</t>
         </is>
       </c>
     </row>
@@ -3740,32 +3744,32 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>96</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>TABLE 95: AVERAGE PREMIUM INCOME PER POLICY FOR INDIVIDUAL AND CORPORATE AGENTS</t>
+          <t>TABLE 96: INSURER-WISE STATE-WISE DISTRIBUTION OF INDIVIDUAL AGENTS OF LIFE INSURERS</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports</t>
+          <t>State-wise</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>Statements &amp; Reports → pick Insurer → Statement = «Avg Premium per Policy» → Fin Year → Quarter</t>
+          <t>State-wise View → pick State → Line of Business = «Individual Agents (Life)» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>State</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Avg Premium per Policy</t>
+          <t>Individual Agents (Life)</t>
         </is>
       </c>
     </row>
@@ -3777,12 +3781,12 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>97</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>TABLE 96: INSURER-WISE STATE-WISE DISTRIBUTION OF INDIVIDUAL AGENTS OF LIFE INSURERS</t>
+          <t>TABLE 97: STATE-WISE NUMBER OF REGISTERED BROKERS</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -3792,7 +3796,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «Individual Agents (Life)» → Class of Biz → Metric → Fin Year</t>
+          <t>State-wise View → pick State → Line of Business = «All Lines» → Class of Biz → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -3802,7 +3806,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Individual Agents (Life)</t>
+          <t>All Lines</t>
         </is>
       </c>
     </row>
@@ -3814,12 +3818,12 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>98</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>TABLE 97: STATE-WISE NUMBER OF REGISTERED BROKERS</t>
+          <t>TABLE 98: STATE AND UT WISE NUMBER OF INSURANCE MARKETING FIRMS</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -3851,32 +3855,32 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>TABLE 98: STATE AND UT WISE NUMBER OF INSURANCE MARKETING FIRMS</t>
+          <t>TABLE 99: CHANNEL-WISE - LIFE INSURANCE - INDIVIDUAL NEW BUSINESS</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>State-wise</t>
+          <t>Channel-wise</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>State-wise View → pick State → Line of Business = «All Lines» → Class of Biz → Metric → Fin Year</t>
+          <t>Channel-wise View → pick Channel → Line of Business = «Life - Individual New Business» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>All Lines</t>
+          <t>Life - Individual New Business</t>
         </is>
       </c>
     </row>
@@ -3888,12 +3892,12 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>101</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>TABLE 99: CHANNEL-WISE - LIFE INSURANCE - INDIVIDUAL NEW BUSINESS</t>
+          <t>TABLE 101: CHANNEL WISE - LIFE INSURANCE GROUP NEW BUSINESS</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -3903,7 +3907,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Channel-wise View → pick Channel → Line of Business = «Life - Individual New Business» → Metric → Fin Year</t>
+          <t>Channel-wise View → pick Channel → Line of Business = «Life - Group New Business» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -3913,7 +3917,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Life - Individual New Business</t>
+          <t>Life - Group New Business</t>
         </is>
       </c>
     </row>
@@ -3925,12 +3929,12 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>103</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>TABLE 101: CHANNEL WISE - LIFE INSURANCE GROUP NEW BUSINESS</t>
+          <t>TABLE 103: CHANNEL-WISE GENERAL INSURANCE BUSINESS</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -3940,7 +3944,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Channel-wise View → pick Channel → Line of Business = «Life - Group New Business» → Metric → Fin Year</t>
+          <t>Channel-wise View → pick Channel → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -3948,11 +3952,7 @@
           <t>Channel</t>
         </is>
       </c>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>Life - Group New Business</t>
-        </is>
-      </c>
+      <c r="G96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3962,12 +3962,12 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>104</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>TABLE 103: CHANNEL-WISE GENERAL INSURANCE BUSINESS</t>
+          <t>TABLE 104: CHANNEL WISE - HEALTH INSURANCE BUSINESS (EXCLUDING TRAVEL AND PERSONAL ACCIDENT INSURANCE)</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -3977,7 +3977,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Channel-wise View → pick Channel → Line of Business = «the segment (Fire / Marine / Motor / Health / …)» → Metric → Fin Year</t>
+          <t>Channel-wise View → pick Channel → Line of Business = «Health» → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -3985,44 +3985,44 @@
           <t>Channel</t>
         </is>
       </c>
-      <c r="G97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Part V</t>
+          <t>Summary</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>A-C</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>TABLE 104: CHANNEL WISE - HEALTH INSURANCE BUSINESS (EXCLUDING TRAVEL AND PERSONAL ACCIDENT INSURANCE)</t>
+          <t>(sector totals)</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Channel-wise</t>
+          <t>Industry-wise</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Channel-wise View → pick Channel → Line of Business = «Health» → Metric → Fin Year</t>
+          <t>Industry-wise View → pick Sector (Life / General / Indian (All)) → Line of Business → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="G98" s="2" t="inlineStr">
-        <is>
-          <t>Health</t>
-        </is>
-      </c>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4032,63 +4032,30 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>A-C</t>
+          <t>D-E</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>(sector totals)</t>
+          <t>(international reinsurance)</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise</t>
+          <t>Country-wise</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Industry-wise View → pick Sector (Life / General / Indian (All)) → Line of Business → Metric → Fin Year</t>
+          <t>Country-wise View → pick Country → Line of Business → Metric → Fin Year</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Country</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>D-E</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>(international reinsurance)</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>Country-wise</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>Country-wise View → pick Country → Line of Business → Metric → Fin Year</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>